<commit_message>
rice refriferant and solid waste tests
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v01.xlsx
+++ b/Excel/10_SolidWaste_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76CE844-6176-4F80-AA9A-2A17E1254F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB9834F-B764-4EB5-8501-2E7D1FFCEE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="315" yWindow="0" windowWidth="37335" windowHeight="19740" firstSheet="1" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <sheet name="Constants - Solid Waste" sheetId="110" r:id="rId6"/>
     <sheet name="Constants - Common" sheetId="122" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -57,7 +54,9 @@
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1, _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(1, (_xlpm.LookupArray1 = _xlpm.LookupValue1) * (_xlpm.LookupArray2 = _xlpm.LookupValue2), _xlpm.ReturnArray, ""))</definedName>
+    <definedName name="Common_InputFunctions.Utility_ResultsItemFromEquationTitleAndSource">_xlfn.LAMBDA(_xlpm.TitleCell,_xlpm.SourceCell, SUBSTITUTE(LEFT(_xlpm.SourceCell, FIND(",", _xlpm.SourceCell) - 1), "VEERG 2026: ", "") &amp; " " &amp; _xlpm.TitleCell)</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlink">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
+    <definedName name="Common_InputFunctions.Utility_SourceHyperlinkDifferentSheet">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SplitStringIntoArray">_xlfn.LAMBDA(_xlpm.Cell,_xlpm.Delimiter,_xlop.CharacterToRemove1,_xlop.CharacterToRemove2, _xlfn.FILTERXML("&lt;t&gt;&lt;s&gt;" &amp; SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.Cell, _xlpm.CharacterToRemove1, ""), _xlpm.CharacterToRemove2, ""), _xlpm.Delimiter, "&lt;/s&gt;&lt;s&gt;") &amp; "&lt;/s&gt;&lt;/t&gt;", "//s"))</definedName>
     <definedName name="Common_InputFunctions.Utility_SumQuantityFromCriteria">_xlfn.LAMBDA(_xlpm.Criteria1,_xlpm.Criteria1TypeArray,_xlpm.Quantity,_xlop.Multiplier,_xlop.Criteria2,_xlop.Criteria2Array, _xlfn.LET(_xlpm.multiplier, IF(_xlfn.ISOMITTED(_xlpm.Multiplier), 1, _xlpm.Multiplier), _xlpm.quantity, _xlpm.Quantity * _xlpm.multiplier, _xlpm.criteria1, --(_xlpm.Criteria1TypeArray = _xlpm.Criteria1), _xlpm.criteria2, IF(_xlfn.ISOMITTED(_xlpm.Criteria2), 1, --(_xlpm.Criteria2Array = _xlpm.Criteria2)), SUMPRODUCT(_xlpm.criteria1 * _xlpm.criteria2 * _xlpm.quantity)))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State/Territory","Common Name","Abbreviation";"New South Wales","New South Wales","NSW";"Australian Capital Territory","ACT","ACT";"Victoria","Victoria","VIC";"Queensland","Queensland","QLD";"South Australia","South Australia","SA";"Western Australia","Western Australia","WA";"Tasmania","Tasmania","TAS";"Northern Territory","Northern Territory","NT"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -250,12 +249,12 @@
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Unit">_xlfn.LAMBDA("t")</definedName>
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Variable">_xlfn.LAMBDA("Q_wt")</definedName>
     <definedName name="WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment">_xlfn.LAMBDA(_xlpm.TreatmentArray,_xlpm.WasteArray,_xlpm.TreatmentLocationArray,_xlpm.UnitArray,_xlpm.AmountArray,_xlpm.TreatmentType,_xlpm.WasteType,_xlpm.TreatmentLocationType,_xlpm.UnitType, SUMIFS(_xlpm.AmountArray, _xlpm.TreatmentArray, _xlpm.TreatmentType, _xlpm.WasteArray, _xlpm.WasteType, _xlpm.TreatmentLocationArray, _xlpm.TreatmentLocationType, _xlpm.UnitArray, _xlpm.UnitType))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(21, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunnings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert Waste",0.11,"";"Incineration","Municipal Solid Waste",0.0537,"NGAF 2025 Table 18";"Incineration","Industrial Waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(21, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert Waste",0.11,"";"Incineration","Municipal Solid Waste",0.0537,"NGAF 2025 Table 18";"Incineration","Industrial Waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.1"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Title">_xlfn.LAMBDA(("Emission factors for wastes disposed of at different treatment facilities"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Unit">_xlfn.LAMBDA(("t CO2e / t"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variable">_xlfn.LAMBDA(("EFwt"))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variation">_xlfn.LAMBDA(("VARIATION ON SOURCE: Fixed typo 'paper and carboard' to 'paper and cardboard'. Added EF source column with specific references."))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variation">_xlfn.LAMBDA(("VARIATION ON SOURCE: Fixed typo 'paper and carboard' to 'paper and cardboard'.  Fixed typo 'prunnings' to 'prunings'. Added EF source column with specific references."))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(12, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Waste type w","VTMw";"Food waste (including animal carcasses, spoiled animal feed or crop)",0.5;"Paper and cardboard",0.09;"Green waste (including crop residues or prunings)",0.24;"Wood",0.15;"Textiles",0.14;"Sludge",0.72;"Rubber and leather",0.14;"Inert waste (including concrete, metal, plastic or glass)",0.42;"Municipal solid waste",0.36;"Commercial and industrial waste",0.33;"Construction and demolition waste",0.39}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.2"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Title">_xlfn.LAMBDA(("Volume to mass conversion factor for various waste types"))</definedName>
@@ -321,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="156">
   <si>
     <t>Home</t>
   </si>
@@ -692,9 +691,6 @@
   </si>
   <si>
     <t>Solid waste treatment</t>
-  </si>
-  <si>
-    <t>Burn all the cardboard</t>
   </si>
   <si>
     <t>Treated on-site</t>
@@ -781,6 +777,63 @@
   </si>
   <si>
     <t>10: Solid Waste Treatment: Results</t>
+  </si>
+  <si>
+    <t>Burn all the cardboard somewhere else</t>
+  </si>
+  <si>
+    <t>Composting</t>
+  </si>
+  <si>
+    <t>All organic waste</t>
+  </si>
+  <si>
+    <t>Compost on-site</t>
+  </si>
+  <si>
+    <t>Burn all the cardboard somewhere else again</t>
+  </si>
+  <si>
+    <t>Compost on site again</t>
+  </si>
+  <si>
+    <t>Landfill food waste on site (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill food waste on site (m3)</t>
+  </si>
+  <si>
+    <t>Landfill food waste offsite (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill food waste offsite (m3)</t>
+  </si>
+  <si>
+    <t>Green waste (including crop residues or prunnings)</t>
+  </si>
+  <si>
+    <t>Landfill Paper offsite (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill Paper waste offsite (m3)</t>
+  </si>
+  <si>
+    <t>Landfill Paper waste on site (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill Paper on site (m3)</t>
+  </si>
+  <si>
+    <t>Landfill Green waste offsite (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill Green waste offsite (m3)</t>
+  </si>
+  <si>
+    <t>Landfill Green waste on site (tonnes)</t>
+  </si>
+  <si>
+    <t>Landfill Green waste on site (m3)</t>
   </si>
 </sst>
 </file>
@@ -1637,7 +1690,7 @@
     </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1852,6 +1905,9 @@
     <xf numFmtId="0" fontId="45" fillId="4" borderId="2" xfId="64">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="56" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="67">
     <cellStyle name="Alert" xfId="59" xr:uid="{34EFE908-8095-4010-8F93-8CFE88055637}"/>
@@ -1923,6 +1979,292 @@
     <cellStyle name="Variable type other" xfId="63" xr:uid="{6646F6F7-E4F9-4165-8015-E25083532B5B}"/>
   </cellStyles>
   <dxfs count="72">
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC44340"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2779,292 +3121,6 @@
         <name val="Times New Roman"/>
         <family val="2"/>
         <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC44340"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <family val="2"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -4143,27 +4199,51 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>48308</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>171886</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{614E1796-C1F6-2C5A-19B2-16B77FB0A30F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16173450" y="5105400"/>
+          <a:ext cx="4896533" cy="3124636"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Acknowledgements"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4231,8 +4311,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AB3DA401-69B9-4F52-A3AF-08FA63C556A0}" name="Table_Input_SolidWaste" displayName="Table_Input_SolidWaste" ref="D9:I18" totalsRowShown="0" headerRowCellStyle="Input table column header">
-  <autoFilter ref="D9:I18" xr:uid="{AB3DA401-69B9-4F52-A3AF-08FA63C556A0}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AB3DA401-69B9-4F52-A3AF-08FA63C556A0}" name="Table_Input_SolidWaste" displayName="Table_Input_SolidWaste" ref="D9:I31" totalsRowShown="0" headerRowCellStyle="Input table column header">
+  <autoFilter ref="D9:I31" xr:uid="{AB3DA401-69B9-4F52-A3AF-08FA63C556A0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -4324,49 +4404,49 @@
     <tableColumn id="1" xr3:uid="{A2B430F3-D1CF-4DBE-B788-FF3C20E22F28}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3CDDB25-5D60-4029-A9DA-FCDF6DED306F}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{C3CDDB25-5D60-4029-A9DA-FCDF6DED306F}" name="MAT" totalsRowDxfId="59" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9679764B-2260-453C-903D-6DDFD533890A}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{9679764B-2260-453C-903D-6DDFD533890A}" name="MAP" totalsRowDxfId="58" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E0B96EC6-4CC7-4E17-A726-BE318859D69B}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{E0B96EC6-4CC7-4E17-A726-BE318859D69B}" name="Frost days per year" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{99D9532F-D633-43D8-9E09-E4CDFE2DA99A}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{99D9532F-D633-43D8-9E09-E4CDFE2DA99A}" name="Elevation" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8EE4536F-60D5-4869-942F-180544702200}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{8EE4536F-60D5-4869-942F-180544702200}" name="MAP:PET" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{0FBAF10F-60EE-41D9-8B7E-87B685FD0BCF}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{0FBAF10F-60EE-41D9-8B7E-87B685FD0BCF}" name="Min temp" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{AAFC57CF-79ED-4BE2-8E90-4DD13CE49372}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{AAFC57CF-79ED-4BE2-8E90-4DD13CE49372}" name="Max temp" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{957B0523-D24F-4CDC-962F-4D2B1660898D}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{957B0523-D24F-4CDC-962F-4D2B1660898D}" name="Min rainfall" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{9E77BCDD-0E8C-4CF0-A1C5-85B308D8C052}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{9E77BCDD-0E8C-4CF0-A1C5-85B308D8C052}" name="Max rainfall" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{153CE395-CEED-4627-A2F5-BCEAC4C343B6}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{153CE395-CEED-4627-A2F5-BCEAC4C343B6}" name="Min frost days" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{AF3247BE-0748-4077-A088-B88274EDB78C}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{AF3247BE-0748-4077-A088-B88274EDB78C}" name="Max frost days" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{CA08E02B-2B67-4F32-A544-1CD765406C64}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{CA08E02B-2B67-4F32-A544-1CD765406C64}" name="Min elevation" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{C508455B-0B90-439D-B21C-483306D70F51}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{C508455B-0B90-439D-B21C-483306D70F51}" name="Max elevation" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{0F2F2640-788C-4191-ACF6-E8907F671213}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{0F2F2640-788C-4191-ACF6-E8907F671213}" name="Min MAP:PET" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{3886FF95-FFB6-4E58-8C4E-685D6C6DD1F1}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{3886FF95-FFB6-4E58-8C4E-685D6C6DD1F1}" name="Max MAP:PET" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4384,7 +4464,7 @@
     <tableColumn id="1" xr3:uid="{82668848-C846-4A8E-BEB5-6A099515513D}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F02B3268-15E1-4043-8BFA-C290D5EDE873}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{F02B3268-15E1-4043-8BFA-C290D5EDE873}" name="Wet or Dry Zone" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4490,7 +4570,7 @@
     <tableColumn id="1" xr3:uid="{A87C906C-828A-4DE3-9EB3-2FCA8EE8054D}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D7930F92-DBDF-4FD8-BF44-B4D67BB114A7}" name="FracWET" dataDxfId="19">
+    <tableColumn id="2" xr3:uid="{D7930F92-DBDF-4FD8-BF44-B4D67BB114A7}" name="FracWET" dataDxfId="43">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4540,13 +4620,13 @@
     <tableColumn id="1" xr3:uid="{27ECD0A0-9936-4A60-BCC5-02F0C62FDA6C}" name="Treatment type t">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="59" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B7AF1F5E-7BAC-4FF7-B59E-F905655514F2}" name="Waste type w" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="58" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{EEC6B364-DA50-41AA-A530-330FAEE98233}" name="EFwt" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="57" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{01FD94D2-85D3-4478-AB5E-04E4027C2978}" name="EF source" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4564,7 +4644,7 @@
     <tableColumn id="1" xr3:uid="{A399DD2C-2C8F-4921-AE90-4A605954450F}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4E1AF06C-CDE4-4181-A993-5B0147FA6DF4}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{4E1AF06C-CDE4-4181-A993-5B0147FA6DF4}" name="FracWET" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4582,7 +4662,7 @@
     <tableColumn id="1" xr3:uid="{34C2D9DB-EED2-456F-BEA2-E59493B21593}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D0EDC8DD-395C-467A-B621-EFC3308C0D3A}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{D0EDC8DD-395C-467A-B621-EFC3308C0D3A}" name="EFPRP" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4600,7 +4680,7 @@
     <tableColumn id="1" xr3:uid="{4295FB4A-FD24-4CF1-93B7-91D96C60BA18}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8C39FACA-411D-4F92-BE74-1F43448F529F}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{8C39FACA-411D-4F92-BE74-1F43448F529F}" name="Season" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4632,49 +4712,49 @@
     <tableColumn id="1" xr3:uid="{4888068E-C9B5-43FD-A916-9B7704914745}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B0FC6643-2FC3-4D44-9372-A36B5CC73DD7}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B0FC6643-2FC3-4D44-9372-A36B5CC73DD7}" name="MAT (ºC)" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0E51BB47-0324-4B13-8E89-7C9A5A09EC52}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{0E51BB47-0324-4B13-8E89-7C9A5A09EC52}" name="Anaerobic lagoon" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2312BF22-4881-442C-A8FD-F976FFCB79B7}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{2312BF22-4881-442C-A8FD-F976FFCB79B7}" name="Digester / covered lagoons" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{1B70D6DD-C0F4-4284-8B69-FAEF867F1C6E}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{1B70D6DD-C0F4-4284-8B69-FAEF867F1C6E}" name="Liquid systems" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{2D0359C8-B312-4F0D-95CC-9F27DD9711CE}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{2D0359C8-B312-4F0D-95CC-9F27DD9711CE}" name="Daily spread" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5A63BD27-4E04-4451-82B2-4721FC78703D}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{5A63BD27-4E04-4451-82B2-4721FC78703D}" name="Composting (passive windrow)" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9E6852C8-02EF-45CF-AE8F-A903AAB60C57}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{9E6852C8-02EF-45CF-AE8F-A903AAB60C57}" name="Solid storage" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{74FF0616-5C4C-44A7-B4AB-CD29BC2285D1}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{74FF0616-5C4C-44A7-B4AB-CD29BC2285D1}" name="Pit storage" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{DC8F4831-78E1-4196-A054-44C26274DAB4}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{DC8F4831-78E1-4196-A054-44C26274DAB4}" name="Deep litter" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F4FFBAFB-4252-464A-913F-2B9A9D6C2256}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{F4FFBAFB-4252-464A-913F-2B9A9D6C2256}" name="Poultry manure with bedding" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{9563BB03-86A6-4D44-AA7D-D448DA9F57D7}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{9563BB03-86A6-4D44-AA7D-D448DA9F57D7}" name="Poultry manure without bedding" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{E7174980-0D39-4A0A-8B4A-73861E176A7D}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{E7174980-0D39-4A0A-8B4A-73861E176A7D}" name="Direct processing" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{DD03C9E8-98A5-4484-920C-D6CF9FB7836F}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{DD03C9E8-98A5-4484-920C-D6CF9FB7836F}" name="Direct application" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{AFBD0566-0721-4CC3-A56B-684599A1581B}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{AFBD0566-0721-4CC3-A56B-684599A1581B}" name="Pasture range and paddock" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{25C1DBBE-A111-4ED1-ABEE-B8DF2C7A1776}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{25C1DBBE-A111-4ED1-ABEE-B8DF2C7A1776}" name="MAT raw" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4692,7 +4772,7 @@
     <tableColumn id="1" xr3:uid="{E51F1B45-76B8-41BA-A4E8-39E28B5D22D8}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1C4AE05B-BAAC-4518-B0E9-FA3DAFBD52CD}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{1C4AE05B-BAAC-4518-B0E9-FA3DAFBD52CD}" name="EFNi &amp; EFN2Oi" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4710,7 +4790,7 @@
     <tableColumn id="1" xr3:uid="{E899A810-DA34-4DD3-9420-7017118A50BC}" name="Waste type w">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{EC8E9200-43B6-459C-B7A6-907C4A1A3CDE}" name="VTMw" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data(), Table_SourceData_WasteSolid_VolumeToMassConversion[[#Headers],[Waste type w]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4733,7 +4813,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K9:K16" totalsRowShown="0" headerRowDxfId="55" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}" name="Table_WasteTypes_Incineration" displayName="Table_WasteTypes_Incineration" ref="K9:K16" totalsRowShown="0" headerRowDxfId="19" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="K9:K16" xr:uid="{9A900595-7035-4239-9059-ACC16835BF72}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -4747,7 +4827,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M9:M10" totalsRowShown="0" headerRowDxfId="54" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}" name="Table_WasteTypes_Composting" displayName="Table_WasteTypes_Composting" ref="M9:M10" totalsRowShown="0" headerRowDxfId="18" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="M9:M10" xr:uid="{5C8D39D3-1330-49EB-B431-1B2B8C8238DC}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -4761,7 +4841,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O9:O10" totalsRowShown="0" headerRowDxfId="53" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}" name="Table_WasteTypes_Anaerobicdigestion" displayName="Table_WasteTypes_Anaerobicdigestion" ref="O9:O10" totalsRowShown="0" headerRowDxfId="17" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="O9:O10" xr:uid="{331EC43E-DF68-429F-A2A4-58BFE6216EC3}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
@@ -5033,7 +5113,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="831" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="803" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5095,7 +5175,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D1" s="55"/>
       <c r="E1" s="55"/>
@@ -5305,7 +5385,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="54" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -5396,15 +5476,15 @@
       <c r="A9" s="13"/>
       <c r="C9" s="18"/>
       <c r="D9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E9" s="53">
         <f>'10.1.1-2 Solid waste treatment'!E109</f>
-        <v>210.92105000000001</v>
+        <v>339.65000000000003</v>
       </c>
       <c r="F9" s="53">
         <f>E9</f>
-        <v>210.92105000000001</v>
+        <v>339.65000000000003</v>
       </c>
       <c r="G9" s="30" t="s">
         <v>58</v>
@@ -5438,7 +5518,7 @@
       <c r="A12" s="13"/>
       <c r="C12" s="18"/>
       <c r="D12" s="39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E12" s="39" t="s">
         <v>60</v>
@@ -5457,15 +5537,15 @@
       </c>
       <c r="C13" s="18"/>
       <c r="D13" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E13" s="53">
         <f>'10.1.1-2 Solid waste treatment'!E136</f>
-        <v>158.42105000000001</v>
+        <v>338.27105</v>
       </c>
       <c r="F13" s="53">
         <f>E13</f>
-        <v>158.42105000000001</v>
+        <v>338.27105</v>
       </c>
       <c r="G13" s="30" t="s">
         <v>58</v>
@@ -6082,7 +6162,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC610A2-02A7-4F78-A2BB-B4DFE856D1FB}">
-  <dimension ref="A1:L371"/>
+  <dimension ref="A1:L384"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -6180,13 +6260,13 @@
         <v>45</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="E10" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="27" t="s">
         <v>117</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>118</v>
       </c>
       <c r="G10" s="27" t="s">
         <v>112</v>
@@ -6203,15 +6283,17 @@
         <f>HYPERLINK("#'10.1.1-2 Solid waste treatment'!A1", "10.1.1-2 Solid waste treatment")</f>
         <v>10.1.1-2 Solid waste treatment</v>
       </c>
-      <c r="D11" s="26"/>
+      <c r="D11" s="26" t="s">
+        <v>140</v>
+      </c>
       <c r="E11" s="27" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H11" s="75">
         <v>50</v>
@@ -6222,12 +6304,14 @@
     </row>
     <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
-      <c r="D12" s="26"/>
+      <c r="D12" s="26" t="s">
+        <v>141</v>
+      </c>
       <c r="E12" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="F12" s="27" t="s">
         <v>117</v>
-      </c>
-      <c r="F12" s="27" t="s">
-        <v>118</v>
       </c>
       <c r="G12" s="27" t="s">
         <v>112</v>
@@ -6243,15 +6327,17 @@
       <c r="A13" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="26"/>
+      <c r="D13" s="26" t="s">
+        <v>142</v>
+      </c>
       <c r="E13" s="27" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H13" s="75">
         <v>50</v>
@@ -6265,12 +6351,14 @@
         <f>HYPERLINK("#'Constants - Solid waste'!A1", "Constants - Solid waste")</f>
         <v>Constants - Solid waste</v>
       </c>
-      <c r="D14" s="26"/>
+      <c r="D14" s="26" t="s">
+        <v>145</v>
+      </c>
       <c r="E14" s="27" t="s">
         <v>107</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G14" s="27" t="s">
         <v>112</v>
@@ -6279,7 +6367,7 @@
         <v>50</v>
       </c>
       <c r="I14" s="27" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6287,15 +6375,17 @@
         <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
         <v>Constants - Common</v>
       </c>
-      <c r="D15" s="26"/>
+      <c r="D15" s="26" t="s">
+        <v>146</v>
+      </c>
       <c r="E15" s="27" t="s">
         <v>107</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H15" s="75">
         <v>50</v>
@@ -6305,15 +6395,17 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="26"/>
+      <c r="D16" s="26" t="s">
+        <v>143</v>
+      </c>
       <c r="E16" s="27" t="s">
         <v>107</v>
       </c>
       <c r="F16" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H16" s="75">
         <v>50</v>
@@ -6323,67 +6415,240 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="26"/>
+      <c r="D17" s="26" t="s">
+        <v>144</v>
+      </c>
       <c r="E17" s="27" t="s">
         <v>107</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H17" s="75">
         <v>50</v>
       </c>
       <c r="I17" s="27" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="26"/>
+      <c r="D18" s="26" t="s">
+        <v>148</v>
+      </c>
       <c r="E18" s="27" t="s">
         <v>107</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="G18" s="27" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H18" s="75">
         <v>50</v>
       </c>
       <c r="I18" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="E19" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="H19" s="75">
+        <v>50</v>
+      </c>
+      <c r="I19" s="27" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
+      <c r="D20" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" s="75">
+        <v>50</v>
+      </c>
+      <c r="I20" s="27" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
-    </row>
-    <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D21" s="26" t="s">
+        <v>151</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="75">
+        <v>50</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D22" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F22" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="75">
+        <v>50</v>
+      </c>
+      <c r="I22" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
     <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
-    </row>
-    <row r="24" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="D23" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F23" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="G23" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="H23" s="75">
+        <v>50</v>
+      </c>
+      <c r="I23" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D24" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="G24" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="H24" s="75">
+        <v>50</v>
+      </c>
+      <c r="I24" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D25" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="G25" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="H25" s="75">
+        <v>50</v>
+      </c>
+      <c r="I25" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D26" s="26"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="77"/>
+      <c r="I26" s="27"/>
+    </row>
+    <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D27" s="26"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="77"/>
+      <c r="I27" s="27"/>
+    </row>
+    <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D28" s="26"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="77"/>
+      <c r="I28" s="27"/>
+    </row>
     <row r="29" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="77"/>
+      <c r="I29" s="27"/>
       <c r="K29" s="47"/>
     </row>
     <row r="30" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="77"/>
+      <c r="I30" s="27"/>
       <c r="K30" s="47"/>
     </row>
     <row r="31" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="77"/>
+      <c r="I31" s="27"/>
       <c r="K31" s="47"/>
     </row>
     <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6445,44 +6710,44 @@
     <row r="46" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="47" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D59" s="66"/>
-    </row>
-    <row r="60" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D61" s="66"/>
-    </row>
-    <row r="62" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D62" s="66"/>
-    </row>
-    <row r="63" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D72" s="66"/>
+    </row>
+    <row r="73" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D74" s="66"/>
+    </row>
+    <row r="75" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D75" s="66"/>
+    </row>
+    <row r="76" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="81" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="82" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6568,121 +6833,121 @@
     <row r="163" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="164" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="165" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="371" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D371" s="38"/>
+    <row r="384" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D384" s="38"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F148:F149">
-    <cfRule type="cellIs" dxfId="52" priority="20" operator="lessThan">
+  <conditionalFormatting sqref="F161:F162">
+    <cfRule type="cellIs" dxfId="16" priority="20" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F160:F161">
-    <cfRule type="cellIs" dxfId="51" priority="19" operator="lessThan">
+  <conditionalFormatting sqref="F173:F174">
+    <cfRule type="cellIs" dxfId="15" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F172:F173">
-    <cfRule type="cellIs" dxfId="50" priority="18" operator="lessThan">
+  <conditionalFormatting sqref="F185:F186">
+    <cfRule type="cellIs" dxfId="14" priority="18" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F260:F261">
-    <cfRule type="cellIs" dxfId="49" priority="93" operator="lessThan">
+  <conditionalFormatting sqref="F273:F274">
+    <cfRule type="cellIs" dxfId="13" priority="93" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F265:F266">
-    <cfRule type="cellIs" dxfId="48" priority="92" operator="lessThan">
+  <conditionalFormatting sqref="F278:F279">
+    <cfRule type="cellIs" dxfId="12" priority="92" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F270:F271">
-    <cfRule type="cellIs" dxfId="47" priority="91" operator="lessThan">
+  <conditionalFormatting sqref="F283:F284">
+    <cfRule type="cellIs" dxfId="11" priority="91" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F294:F295">
-    <cfRule type="cellIs" dxfId="46" priority="85" operator="lessThan">
+  <conditionalFormatting sqref="F307:F308">
+    <cfRule type="cellIs" dxfId="10" priority="85" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F299:F300">
-    <cfRule type="cellIs" dxfId="45" priority="84" operator="lessThan">
+  <conditionalFormatting sqref="F312:F313">
+    <cfRule type="cellIs" dxfId="9" priority="84" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F304:F305">
-    <cfRule type="cellIs" dxfId="44" priority="83" operator="lessThan">
+  <conditionalFormatting sqref="F317:F318">
+    <cfRule type="cellIs" dxfId="8" priority="83" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I19 F57">
-    <cfRule type="cellIs" dxfId="43" priority="62" operator="lessThan">
+  <conditionalFormatting sqref="I32 F70">
+    <cfRule type="cellIs" dxfId="7" priority="62" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I65:I69">
-    <cfRule type="cellIs" dxfId="42" priority="5" operator="lessThan">
+  <conditionalFormatting sqref="I78:I82">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I73 I132">
-    <cfRule type="cellIs" dxfId="41" priority="74" operator="lessThan">
+  <conditionalFormatting sqref="I86 I145">
+    <cfRule type="cellIs" dxfId="5" priority="74" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I84:I86">
-    <cfRule type="cellIs" dxfId="40" priority="4" operator="lessThan">
+  <conditionalFormatting sqref="I97:I99">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I90:I93">
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="I103:I106">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I97:I101">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="lessThan">
+  <conditionalFormatting sqref="I110:I114">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J8 I51:I52 H53:H55 I54 I56:I58 I60:I61 I212 I218 E220:G220">
-    <cfRule type="cellIs" dxfId="37" priority="79" operator="lessThan">
+  <conditionalFormatting sqref="J8 I64:I65 H66:H68 I67 I69:I71 I73:I74 I225 I231 E233:G233">
+    <cfRule type="cellIs" dxfId="1" priority="79" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J37 I45 F136:F137">
-    <cfRule type="cellIs" dxfId="36" priority="21" operator="lessThan">
+  <conditionalFormatting sqref="J37 I58 F149:F150">
+    <cfRule type="cellIs" dxfId="0" priority="21" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D287" xr:uid="{4E913AB3-F90B-4C35-BCE1-5DBB8FC05107}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D300" xr:uid="{4E913AB3-F90B-4C35-BCE1-5DBB8FC05107}">
       <formula1>INDIRECT("Table_SourceData_PoultryMMSStage1[MMS]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E235" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E248" xr:uid="{9FB53635-991F-44AA-A123-E8ABEF9EE0A6}">
       <formula1>INDIRECT("Table_SourceData_Dairy_ProductionSystemTemplates[Area]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E259 E264 E269 E303 E298 E293 E171 E159 E135 E147" xr:uid="{00A4EA4C-90D3-4150-979D-4D71C7F37A31}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E272 E277 E282 E316 E311 E306 E184 E172 E148 E160" xr:uid="{00A4EA4C-90D3-4150-979D-4D71C7F37A31}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E75" xr:uid="{DBA884B0-B52E-420E-8FD2-21B082EB75E2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E88" xr:uid="{DBA884B0-B52E-420E-8FD2-21B082EB75E2}">
       <formula1>INDIRECT("Table_SourceData_Swine_IrrigationMethods[Irrigation method]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E21" xr:uid="{48A1E533-1334-4AAC-A5F5-B295A34573CB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E34" xr:uid="{48A1E533-1334-4AAC-A5F5-B295A34573CB}">
       <formula1>INDIRECT("Table_SourceData_ElectricityEFs[State, Territory or grid description]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E18" xr:uid="{BE2CA0F8-93F9-493C-B304-DCA372760E4E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E31" xr:uid="{BE2CA0F8-93F9-493C-B304-DCA372760E4E}">
       <formula1>INDIRECT(_xlfn.UNIQUE("Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t]"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:G18" xr:uid="{EB782CB2-069D-4346-96A4-9C640517727F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:G31" xr:uid="{EB782CB2-069D-4346-96A4-9C640517727F}">
       <formula1>"Treated on-site, Removed and treated off-site"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I10:I18" xr:uid="{5637D9FB-43C0-46B6-8C23-E9E5D77EE5AE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I10:I31" xr:uid="{5637D9FB-43C0-46B6-8C23-E9E5D77EE5AE}">
       <formula1>"tonnes, cubic metres m3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F18" xr:uid="{502FA925-EB70-4F2C-8CD1-14FB9D0D2E6F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F31" xr:uid="{502FA925-EB70-4F2C-8CD1-14FB9D0D2E6F}">
       <formula1>INDIRECT("Table_WasteTypes_" &amp; SUBSTITUTE(E10, " ", "") &amp; "[Waste type w]")</formula1>
     </dataValidation>
   </dataValidations>
@@ -6918,12 +7183,12 @@
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D18" s="70" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="71" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6958,7 +7223,7 @@
       <c r="F21" s="73"/>
       <c r="G21" s="28" cm="1">
         <f t="array" ref="G21">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D21,E21, "Treated on-site", "cubic metres m3")</f>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H21" s="28" cm="1">
         <f t="array" ref="H21">Common_InputFunctions.Utility_LookupValueInTableNumber(E21,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
@@ -6966,7 +7231,7 @@
       </c>
       <c r="I21" s="28" cm="1">
         <f t="array" ref="I21">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G21,H21)</f>
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6979,7 +7244,7 @@
       <c r="F22" s="73"/>
       <c r="G22" s="28" cm="1">
         <f t="array" ref="G22">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D22,E22, "Treated on-site", "cubic metres m3")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H22" s="28" cm="1">
         <f t="array" ref="H22">Common_InputFunctions.Utility_LookupValueInTableNumber(E22,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
@@ -6987,7 +7252,7 @@
       </c>
       <c r="I22" s="28" cm="1">
         <f t="array" ref="I22">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G22,H22)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6996,7 +7261,7 @@
         <v>Landfill</v>
       </c>
       <c r="E23" s="51" t="str">
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="F23" s="73"/>
       <c r="G23" s="28" cm="1">
@@ -7005,7 +7270,7 @@
       </c>
       <c r="H23" s="28" cm="1">
         <f t="array" ref="H23">Common_InputFunctions.Utility_LookupValueInTableNumber(E23,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I23" s="28" cm="1">
         <f t="array" ref="I23">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G23,H23)</f>
@@ -7211,7 +7476,7 @@
       <c r="F33" s="73"/>
       <c r="G33" s="28" cm="1">
         <f t="array" ref="G33">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D33,E33, "Treated on-site", "cubic metres m3")</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H33" s="28" cm="1">
         <f t="array" ref="H33">Common_InputFunctions.Utility_LookupValueInTableNumber(E33,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
@@ -7219,7 +7484,7 @@
       </c>
       <c r="I33" s="28" cm="1">
         <f t="array" ref="I33">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G33,H33)</f>
-        <v>4.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7337,7 +7602,7 @@
       <c r="F39" s="73"/>
       <c r="G39" s="28" cm="1">
         <f t="array" ref="G39">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D39,E39, "Treated on-site", "cubic metres m3")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H39" s="28" cm="1">
         <f t="array" ref="H39">Common_InputFunctions.Utility_LookupValueInTableNumber(E39,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
@@ -7372,12 +7637,12 @@
     <row r="41" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D42" s="70" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D43" s="71" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="44" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7431,7 +7696,7 @@
       <c r="F46" s="73"/>
       <c r="G46" s="28" cm="1">
         <f t="array" ref="G46">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D46,E46, "Removed and treated off-site", "cubic metres m3")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H46" s="28" cm="1">
         <f t="array" ref="H46">Common_InputFunctions.Utility_LookupValueInTableNumber(E46,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
@@ -7439,7 +7704,7 @@
       </c>
       <c r="I46" s="28" cm="1">
         <f t="array" ref="I46">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G46,H46)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="47" spans="4:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7447,7 +7712,7 @@
         <v>Landfill</v>
       </c>
       <c r="E47" s="51" t="str">
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="F47" s="73"/>
       <c r="G47" s="28" cm="1">
@@ -7456,7 +7721,7 @@
       </c>
       <c r="H47" s="28" cm="1">
         <f t="array" ref="H47">Common_InputFunctions.Utility_LookupValueInTableNumber(E47,Table_SourceData_WasteSolid_VolumeToMassConversion[Waste type w],Table_SourceData_WasteSolid_VolumeToMassConversion[VTMw])</f>
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="I47" s="28" cm="1">
         <f t="array" ref="I47">WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume(G47,H47)</f>
@@ -8004,12 +8269,12 @@
     <row r="84" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="85" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D85" s="70" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="86" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D86" s="71" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="87" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8021,19 +8286,19 @@
       </c>
       <c r="F87" s="67"/>
       <c r="G87" s="67" t="s">
+        <v>126</v>
+      </c>
+      <c r="H87" s="72" t="s">
         <v>127</v>
-      </c>
-      <c r="H87" s="72" t="s">
-        <v>128</v>
       </c>
       <c r="I87" s="72" t="s">
         <v>97</v>
       </c>
       <c r="J87" s="72" t="s">
+        <v>120</v>
+      </c>
+      <c r="K87" s="72" t="s">
         <v>121</v>
-      </c>
-      <c r="K87" s="72" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="88" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8052,11 +8317,11 @@
       </c>
       <c r="H88" s="28">
         <f t="shared" ref="H88:H107" si="0">I21</f>
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I88" s="28">
         <f>G88+H88</f>
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="J88" s="28" cm="1">
         <f t="array" ref="J88">Common_InputFunctions.Utility_LookupValueInTableTwoColumns(D88,E88,Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t],Table_SourceData_WasteSolid_WasteTreatmentEFs[Waste type w],Table_SourceData_WasteSolid_WasteTreatmentEFs[EFwt])</f>
@@ -8064,7 +8329,7 @@
       </c>
       <c r="K88" s="28" cm="1">
         <f t="array" ref="K88">WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement(I88, J88)</f>
-        <v>210</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="89" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8077,15 +8342,15 @@
       <c r="F89" s="73"/>
       <c r="G89" s="28" cm="1">
         <f t="array" ref="G89">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D22,E22, "Treated on-site", "tonnes")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H89" s="28">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I89" s="28">
         <f t="shared" ref="I89:I107" si="1">G89+H89</f>
-        <v>0</v>
+        <v>54.5</v>
       </c>
       <c r="J89" s="28" cm="1">
         <f t="array" ref="J89">Common_InputFunctions.Utility_LookupValueInTableTwoColumns(D89,E89,Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t],Table_SourceData_WasteSolid_WasteTreatmentEFs[Waste type w],Table_SourceData_WasteSolid_WasteTreatmentEFs[EFwt])</f>
@@ -8093,7 +8358,7 @@
       </c>
       <c r="K89" s="28" cm="1">
         <f t="array" ref="K89">WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement(I89, J89)</f>
-        <v>0</v>
+        <v>179.85</v>
       </c>
     </row>
     <row r="90" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8101,7 +8366,7 @@
         <v>Landfill</v>
       </c>
       <c r="E90" s="51" t="str">
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="F90" s="73"/>
       <c r="G90" s="28" cm="1">
@@ -8396,15 +8661,15 @@
       <c r="F100" s="73"/>
       <c r="G100" s="28" cm="1">
         <f t="array" ref="G100">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D33,E33, "Treated on-site", "tonnes")</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H100" s="28">
         <f t="shared" si="0"/>
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I100" s="28">
         <f t="shared" si="1"/>
-        <v>54.5</v>
+        <v>0</v>
       </c>
       <c r="J100" s="28" cm="1">
         <f t="array" ref="J100">Common_InputFunctions.Utility_LookupValueInTableTwoColumns(D100,E100,Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t],Table_SourceData_WasteSolid_WasteTreatmentEFs[Waste type w],Table_SourceData_WasteSolid_WasteTreatmentEFs[EFwt])</f>
@@ -8412,7 +8677,7 @@
       </c>
       <c r="K100" s="28" cm="1">
         <f t="array" ref="K100">WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement(I100, J100)</f>
-        <v>0.92104999999999992</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8570,7 +8835,7 @@
       <c r="F106" s="73"/>
       <c r="G106" s="28" cm="1">
         <f t="array" ref="G106">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D39,E39, "Treated on-site", "tonnes")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H106" s="28">
         <f t="shared" si="0"/>
@@ -8578,7 +8843,7 @@
       </c>
       <c r="I106" s="28">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J106" s="28" cm="1">
         <f t="array" ref="J106">Common_InputFunctions.Utility_LookupValueInTableTwoColumns(D106,E106,Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t],Table_SourceData_WasteSolid_WasteTreatmentEFs[Waste type w],Table_SourceData_WasteSolid_WasteTreatmentEFs[EFwt])</f>
@@ -8586,7 +8851,7 @@
       </c>
       <c r="K106" s="28" cm="1">
         <f t="array" ref="K106">WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement(I106, J106)</f>
-        <v>0</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8625,11 +8890,11 @@
         <v>▲ Back to top</v>
       </c>
       <c r="D109" s="62" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E109" s="64">
         <f>SUM(K88:K107)</f>
-        <v>210.92105000000001</v>
+        <v>339.65000000000003</v>
       </c>
       <c r="F109" s="69" t="str">
         <f>$E$75</f>
@@ -8640,12 +8905,12 @@
     <row r="111" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="112" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D112" s="70" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="113" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D113" s="71" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="114" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8657,19 +8922,19 @@
       </c>
       <c r="F114" s="67"/>
       <c r="G114" s="67" t="s">
+        <v>126</v>
+      </c>
+      <c r="H114" s="72" t="s">
         <v>127</v>
-      </c>
-      <c r="H114" s="72" t="s">
-        <v>128</v>
       </c>
       <c r="I114" s="72" t="s">
         <v>97</v>
       </c>
       <c r="J114" s="72" t="s">
+        <v>120</v>
+      </c>
+      <c r="K114" s="72" t="s">
         <v>121</v>
-      </c>
-      <c r="K114" s="72" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="115" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8713,15 +8978,15 @@
       <c r="F116" s="73"/>
       <c r="G116" s="28" cm="1">
         <f t="array" ref="G116">WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment(Table_Input_SolidWaste[Treatment type (select)],Table_Input_SolidWaste[Waste type (select)],Table_Input_SolidWaste[Treatment location (select)],Table_Input_SolidWaste[Amount unit (select)],Table_Input_SolidWaste[Amount],D22,E22, "Removed and treated off-site", "tonnes")</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H116" s="28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I116" s="28">
         <f t="shared" ref="I116:I134" si="3">G116+H116</f>
-        <v>0</v>
+        <v>54.5</v>
       </c>
       <c r="J116" s="28" cm="1">
         <f t="array" ref="J116">Common_InputFunctions.Utility_LookupValueInTableTwoColumns(D116,E116,Table_SourceData_WasteSolid_WasteTreatmentEFs[Treatment type t],Table_SourceData_WasteSolid_WasteTreatmentEFs[Waste type w],Table_SourceData_WasteSolid_WasteTreatmentEFs[EFwt])</f>
@@ -8729,7 +8994,7 @@
       </c>
       <c r="K116" s="28" cm="1">
         <f t="array" ref="K116">WasteSolid_Equations.VEERG_10_1_1_1__1_EmissionsFromWasteManagement(I116, J116)</f>
-        <v>0</v>
+        <v>179.85</v>
       </c>
     </row>
     <row r="117" spans="4:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -8737,7 +9002,7 @@
         <v>Landfill</v>
       </c>
       <c r="E117" s="51" t="str">
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="F117" s="73"/>
       <c r="G117" s="28" cm="1">
@@ -9261,11 +9526,11 @@
         <v>▲ Back to top</v>
       </c>
       <c r="D136" s="62" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E136" s="64">
         <f>SUM(K115:K134)</f>
-        <v>158.42105000000001</v>
+        <v>338.27105</v>
       </c>
       <c r="F136" s="69" t="str">
         <f>$E$75</f>
@@ -9518,7 +9783,7 @@
       </c>
       <c r="E6" s="31" t="str" cm="1">
         <f t="array" ref="E6">WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variation()</f>
-        <v>VARIATION ON SOURCE: Fixed typo 'paper and carboard' to 'paper and cardboard'. Added EF source column with specific references.</v>
+        <v>VARIATION ON SOURCE: Fixed typo 'paper and carboard' to 'paper and cardboard'.  Fixed typo 'prunnings' to 'prunings'. Added EF source column with specific references.</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -9564,7 +9829,7 @@
         <v>91</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I9" s="26" t="s">
         <v>90</v>
@@ -9654,7 +9919,7 @@
       </c>
       <c r="E12" s="26" t="str" cm="1">
         <f t="array" ref="E12">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="F12" s="26" cm="1">
         <f t="array" ref="F12">Common_InputFunctions.Utility_DisplayArrayInTable(WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data(), Table_SourceData_WasteSolid_WasteTreatmentEFs[[#Headers],[Treatment type t]], 0)</f>
@@ -9666,7 +9931,7 @@
       </c>
       <c r="I12" s="26" t="str">
         <f>Table_SourceData_WasteSolid_WasteTreatmentEFs[[#This Row],[Waste type w]]</f>
-        <v>Green waste (including crop residues or prunnings)</v>
+        <v>Green waste (including crop residues or prunings)</v>
       </c>
       <c r="K12" s="1" t="str">
         <f t="shared" si="0"/>
@@ -14326,15 +14591,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -14343,6 +14599,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14541,24 +14806,24 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQA6ACAAVwBhAHMAdABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAAUwBvAGwAaQBkACAAVwBhAHMAdABlACAAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAbgBFAF8AZwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwBnAD0AXABcAHMAdQBtAF8AdABcAFwAcwB1AG0AXwB3ACgAUQBfAHcAdABcAFwAdABpAG0AZQBzACAARQBGAF8AdwB0AGcAKQBcAG4AUQBfAHcAdAAgAD0AIABxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzACAAKAB0ACkAXABuAEUARgBfAHcAdABnACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAHQAIABDAE8AMgBlAC8AdAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAHcAdAAsACAARQBGAF8AdwB0AGcALABcAG4AIAAgACAAIABRAF8AdwB0ACAAKgAgAEUARgBfAHcAdABnAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAPQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHQAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB3ACgAUQBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAdwB0AGcAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwBcACIALAAgAFwAIgB0AFwAIgAsACAAXAAiAFMAdQBtACAAbwBmACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwB3AHQAZwBcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAHQAIABDAE8AMgBlAC8AdABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwB2AG8AbAB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAHYAbwBsAHUAbQBlACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMQAwAC4AMQAuADEALgAxACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAXwBtAGEAcwBzAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIABtAGEAcwBzAFwAIgAsACAAXAAiAHQAbwBuAG4AZQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAUQBfAHYAbwBsAHcAdAAgAGEAbgBkACAAUQBfAG0AYQBzAHMAdwB0ACAAdgBhAHIAaQBhAGIAbABlAHMAIAB0AG8AIABjAGwAZQBhAHIAbAB5ACAAdAByAGEAYwBrACAAaQBuAHAAdQB0ACAAbwByACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAFEAIAB2AGEAbAB1AGUAcwBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAbgBRAF8AdwB0AFwAbgB0AFwAbgBRAF8AdwB0AD0AVgBfAHcAdABcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAbgBWAF8AdwB0ACAAPQAgAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKABtADMAKQBcAG4AVgBUAE0AXwB3ACAAPQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIAAoAHQALwBtADMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAF8AdwB0ACwAIABWAFQATQBfAHcALABcAG4AIAAgACAAIABWAF8AdwB0ACAAKgAgAFYAVABNAF8AdwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAdwBhAHMAdABlACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAHYAbwBsAHUAbQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHcAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADAALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AewB3AHQAfQA9AFYAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAXwB3AHQAXAAiACwAIABcACIAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAbQAzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBUAE0AXwB3AFwAIgAsACAAXAAiAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAG8AZgAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGYAbwByACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAdAAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHcAXAAiACwAIABcACIAdwBhAHMAdABlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHQAXAAiACwAIABcACIAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB3AGEAcwB0AGUAcwAgAGQAaQBzAHAAbwBzAGUAZAAgAG8AZgAgAGEAdAAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AGkAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUARgB3AHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdABcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAHQAIABDAE8AMgBlACAALwAgAHQAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAxAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAxACwAIAA0ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAdAB5AHAAZQAgAHQAXAAiACwAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIARQBGAHcAdABcACIALAAgAFwAIgBFAEYAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMgAuADEALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADMALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACwAIABnAHIAZQBlAG4AIAB3AGEAcwB0AGUALAAgAHcAbwBvAGQALAAgAHMAbAB1AGQAZwBlAFwAIgAsACAAMAAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAAxADYAOQAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAzADYANgA3ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAwAC4ANAA5ADEAOQAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBlAHIAdAAgAFcAYQBzAHQAZQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABTAG8AbABpAGQAIABXAGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBkAHUAcwB0AHIAaQBhAGwAIABXAGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADQANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAAMgA4ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGIAbwBhAHIAZABcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAB1ADAAMAAyADcALgAgAEEAZABkAGUAZAAgAEUARgAgAHMAbwB1AHIAYwBlACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBwAGUAYwBpAGYAaQBjACAAcgBlAGYAZQByAGUAbgBjAGUAcwAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAOgAgAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwAgACgAdAAvAG0AMwApACAAKABWAFQATQB3ACkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBUAE0AdwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0AC8AbQAzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAVgBUAE0AdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMQA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADcAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADQAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA5AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBoAGEAbgBnAGUAZAAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAIABDAEYAdwAgAHQAbwAgAFYAVABNAHcAIAB0AG8AIABtAGEAdABjAGgAIAB0AGkAdABsAGUAIAB2AGEAcgBpAGEAYgBsAGUALgBcACIAKQApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsACAAVwBhAHMAdABlAFQAeQBwAGUALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABVAG4AaQB0AFQAeQBwAGUALABcAG4AIAAgAFMAVQBNAEkARgBTACgAXABuACAAIAAgACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAXABuACAAIAAgACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFwAbgAgACAAIAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABVAG4AaQB0AFQAeQBwAGUAXABuACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIAAnAEYAcgB5ACcAIAB0AG8AIAAnAEQAcgB5ACcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAD4AIAAxADgAIABDAFwAIgAsACAAXAAiAD4AIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMgAwADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAPgAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAPgAgADAAIABDACAALQAgAGQiIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAZQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAVAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBQACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARQBUACAAPQAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZQB2AGEAcABvAHQAcgBhAG4AcwBwAGkAcgBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAATQBBAFQAIABtAGkAbgAgAGEAbgBkACAATQBBAFQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBlAGQAaQBhAG4AIABBAG4AbgB1AGEAbAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgACgATQBBAFQAKQBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBUAFwAIgAsACAAXAAiAE0AYQB4ACAATQBBAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIgADIANgAgAEMAXAAiACwAIAAyADYALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAXAAiADEANQAgAC0AIAAyADUAIABDAFwAIgAsACAAMQA1ACwAIAAyADUALgA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiIAAxADQAIABDAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQA0AC4AOQA5ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAIABmAHIAbwBtACAAcgBlAGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQAYQB0AGEALgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAFoAbwBuAGUAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIAA+ACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAD4AowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgACcAQQBxAHUAYQBjAHUAbAB0AHUAcgBlACcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQAnACwAIAAnAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAJwAgAGEAbgBkACAAJwBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAJwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlACcAIAByAG8AdwAgAHcAaQB0AGgAIABzAGEAbQBlACAARQBGACAAZgBvAHIAIABsAG8AdwAgAGEAbgBkACAAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBcAG4AVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcAG4ASQBQAEMAQwA6ACAATgAyAE8AIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABNAEEATgBBAEcARQBEACAAUwBPAEkATABTACwAIABBAE4ARAAgAEMATwAyACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATABJAE0ARQAgAEEATgBEACAAVQBSAEUAQQAgAEEAUABQAEwASQBDAEEAVABJAE8ATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAVwBFAFQAIABmAG8AcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgADIAMAAxADkAIABSAGUAZgBpAG4AZQBtAGUAbgB0ACAAVgBvAGwAdQBtAGUAIAA0ADoAIABDAGgAYQBwAHQAZQByACAAMQAxADoAIABOADIATwAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAE0AYQBuAGEAZwBlAGQAIABTAG8AaQBsAHMALAAgAGEAbgBkACAAQwBPADIAIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABMAGkAbQBlACAAYQBuAGQAIABVAHIAZQBhACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAIABpAHIAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHAAcgBpAG4AawBsAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQByAGYAYQBjAGUAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFQAYQBiAGwAZQAgAGMAcgBlAGEAdABlAGQAIABiAGEAcwBlAGQAIABvAG4AIABWAEUARQBSAEcAIAB0AGUAeAB0ACAAJwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgAnAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwAnACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAJwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlACcAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBvAG4AdABoAHMAIAB0AG8AIABTAGUAYQBzAG8AbgBzACAATQBhAHAAcABpAG4AZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwBuAHQAaABcACIALAAgAFwAIgBTAGUAYQBzAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBhAG4AdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGIAcgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAcgBjAGgAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcAByAGkAbABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHkAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBuAGUAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAdQBsAHkAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBnAHUAcwB0AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAcAB0AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwBjAHQAbwBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHYAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAYwBlAG0AYgBlAHIAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgABMgIABNAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAcABlAHIAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADgALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADIALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQBcACIALAAgAFwAIgBNAEEAVAAgACgAugBDACkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBDAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIATABpAHEAdQBpAGQAIABTAGwAdQByAHIAeQAgACgAdwBpAHQAaABvAHUAdAAgAG4AYQB0AHUAcgBhAGwAIABjAHIAdQBzAHQAKQBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZAAgACgAYgApAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBQAGkAdAAgAFMAdABvAHIAYQBnAGUAIAA8ADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIAAnAFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAJwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAZQBwAGEAcgBhAHQAZQAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAAQQBkAGQAZQBkACAAJwBNAEEAVAAgAHIAYQB3ACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBpAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMQAuADQAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAE4AaQAgACYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIAAmACAAXAAiACAAXAAiACAAJgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEAOgAgAFcAYQBzAHQAZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQAwAC4AMQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAFMAbwBsAGkAZAAgAFcAYQBzAHQAZQAgAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdwBhAHMAdABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAGIAeQAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcAG4ARQBfAGcAXABuAHQAIABDAE8AMgBlAFwAbgBFAF8AZwA9AFwAXABzAHUAbQBfAHQAXABcAHMAdQBtAF8AdwAoAFEAXwB3AHQAXABcAHQAaQBtAGUAcwAgAEUARgBfAHcAdABnACkAXABuAFEAXwB3AHQAIAA9ACAAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAbwBmACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACwAIABvAG4AIABhACAAdwBlAHQAIAB3AGUAaQBnAGgAdAAgAGIAYQBzAGkAcwAgACgAdAApAFwAbgBFAEYAXwB3AHQAZwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAZwAgAGYAbwByACAAdABoAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAbwBmACAAdwBhAHMAdABlACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0ACAAKAB0ACAAQwBPADIAZQAvAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwB3AHQALAAgAEUARgBfAHcAdABnACwAXABuACAAIAAgACAAUQBfAHcAdAAgACoAIABFAEYAXwB3AHQAZwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMQAwAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdwAoAFEAXwB7AHcAdAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AHcAdABnAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAXAAiACwAIABcACIAdABcACIALAAgAFwAIgBTAHUAbQAgAG8AZgAgAFEAXwB2AG8AbAB3AHQAIABhAG4AZAAgAFEAXwBtAGEAcwBzAHcAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AdwB0AGcAXAAiACwAIABcACIAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgB0ACAAQwBPADIAZQAvAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB3AFwAIgAsACAAXAAiAHcAYQBzAHQAZQAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB0AFwAIgAsACAAXAAiAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AdgBvAGwAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGQAIAB3AGEAcwB0AGUAIABpAG4AcAB1AHQAIABhAHMAIAB2AG8AbAB1AG0AZQAgAGEAbgBkACAAYwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIAB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADEAMAAuADEALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AbQBhAHMAcwB3AHQAXAAiACwAIABcACIAcQB1AGEAbgB0AGkAdAB5ACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAbQBhAHMAcwBcACIALAAgAFwAIgB0AG8AbgBuAGUAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAFEAXwB2AG8AbAB3AHQAIABhAG4AZAAgAFEAXwBtAGEAcwBzAHcAdAAgAHYAYQByAGkAYQBiAGwAZQBzACAAdABvACAAYwBsAGUAYQByAGwAeQAgAHQAcgBhAGMAawAgAGkAbgBwAHUAdAAgAG8AcgAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABRACAAdgBhAGwAdQBlAHMAXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBcAG4ATQBhAHMAcwAgAG8AZgAgAHcAYQBzAHQAZQAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIAB2AG8AbAB1AG0AZQBcAG4AUQBfAHcAdABcAG4AdABcAG4AUQBfAHcAdAA9AFYAXwB3AHQAXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcAG4AVgBfAHcAdAAgAD0AIAB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAbQAzACkAXABuAFYAVABNAF8AdwAgAD0AIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABvAGYAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABmAG8AcgAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAKAB0AC8AbQAzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBfAHcAdAAsACAAVgBUAE0AXwB3ACwAXABuACAAIAAgACAAVgBfAHcAdAAgACoAIABWAFQATQBfAHcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAHcAYQBzAHQAZQAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIAB2AG8AbAB1AG0AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB3AHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMQAwAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUQBfAHsAdwB0AH0APQBWAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAAVgBUAE0AXwB3AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAF8AdwB0AFwAIgAsACAAXAAiAHYAbwBsAHUAbQBlACAAbwBmACAAcwBvAGwAaQBkACAAdwBhAHMAdABlACAAdAB5AHAAZQAgAHcAIABiAGUAaQBuAGcAIABzAGUAbgB0ACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABmAGEAYwBpAGwAaQB0AHkAIAB0AFwAIgAsACAAXAAiAG0AMwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAVABNAF8AdwBcACIALAAgAFwAIgBjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABvAGYAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABmAG8AcgAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAHQALwBtADMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB3AFwAIgAsACAAXAAiAHcAYQBzAHQAZQAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB0AFwAIgAsACAAXAAiAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdwBhAHMAdABlAHMAIABkAGkAcwBwAG8AcwBlAGQAIABvAGYAIABhAHQAIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdABpAGUAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdwBhAHMAdABlAHMAIABkAGkAcwBwAG8AcwBlAGQAIABvAGYAIABhAHQAIABkAGkAZgBmAGUAcgBlAG4AdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdABpAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAEYAdwB0AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0ACAAQwBPADIAZQAgAC8AIAB0AFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMQBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMQAsACAANAAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHQAeQBwAGUAIAB0AFwAIgAsACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAEUARgB3AHQAXAAiACwAIABcACIARQBGACAAcwBvAHUAcgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgADIALgAxACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAzAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgADAALgA3ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADIALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADQALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAUgB1AGIAYgBlAHIAIABhAG4AZAAgAGwAZQBhAHQAaABlAHIAXAAiACwAIAAzAC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADEANgA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADMANgA2ADcALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgA0ADkAMQA5ACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGUAcgB0ACAAVwBhAHMAdABlAFwAIgAsACAAMAAuADEAMQAwADAALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAFMAbwBsAGkAZAAgAFcAYQBzAHQAZQBcACIALAAgADAALgAwADUAMwA3ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIASQBuAGQAdQBzAHQAcgBpAGEAbAAgAFcAYQBzAHQAZQBcACIALAAgADEALgA2ADQAOQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADAANAA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIABUAGEAYgBsAGUAIAAxADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAAyADgALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAARgBpAHgAZQBkACAAdAB5AHAAbwAgACcAcABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBiAG8AYQByAGQAJwAgAHQAbwAgACcAcABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZAAnAC4AIAAgAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAnAHAAcgB1AG4AbgBpAG4AZwBzACcAIAB0AG8AIAAnAHAAcgB1AG4AaQBuAGcAcwAnAC4AIABBAGQAZABlAGQAIABFAEYAIABzAG8AdQByAGMAZQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAcABlAGMAaQBmAGkAYwAgAHIAZQBmAGUAcgBlAG4AYwBlAHMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyADoAIABWAG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHYAYQByAGkAbwB1AHMAIAB3AGEAcwB0AGUAIAB0AHkAcABlAHMAIAAoAHQALwBtADMAKQAgACgAVgBUAE0AdwApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAVABNAHcAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAvAG0AMwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAxAC4AMgBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAyACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3AFwAIgAsACAAXAAiAFYAVABNAHcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAMAAuADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAMAAuADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAZQB4AHQAaQBsAGUAcwBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA3ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAHUAYgBiAGUAcgAgAGEAbgBkACAAbABlAGEAdABoAGUAcgBcACIALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgA0ADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbgBpAGMAaQBwAGEAbAAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQBcACIALAAgADAALgAzADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBtAGUAcgBjAGkAYQBsACAAYQBuAGQAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEMAaABhAG4AZwBlAGQAIABjAG8AbAB1AG0AbgAgAGgAZQBhAGQAZQByACAAQwBGAHcAIAB0AG8AIABWAFQATQB3ACAAdABvACAAbQBhAHQAYwBoACAAdABpAHQAbABlACAAdgBhAHIAaQBhAGIAbABlAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABBAG0AbwB1AG4AdABBAHIAcgBhAHkALABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAIABUAHIAZQBhAHQAbQBlAG4AdABMAG8AYwBhAHQAaQBvAG4AVAB5AHAAZQAsACAAVQBuAGkAdABUAHkAcABlACwAXABuACAAIABTAFUATQBJAEYAUwAoAFwAbgAgACAAIAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAIABUAHIAZQBhAHQAbQBlAG4AdABBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AFQAeQBwAGUALABcAG4AIAAgACAAIABXAGEAcwB0AGUAQQByAHIAYQB5ACwAIABXAGEAcwB0AGUAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABcAG4AIAAgACAAIABVAG4AaQB0AEEAcgByAGEAeQAsACAAVQBuAGkAdABUAHkAcABlAFwAbgAgACAAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBEAGEAdABhACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVwBhAHMAdABlAFMAbwBsAGkAZABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAFMAdQBtAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
     <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>